<commit_message>
docs: cahier de recettes complet v2.0 (Excel, 7 feuilles)
Couvre l'ensemble des modifications:
- Lot 1: modification de vente (annulation, attribution, suppression copie)
- Lot 2: moteur de suggestion (regles metier + requetes de controle)
- Lot 3: telephone tiers-payant dans les editions PDF
- Lot 4: telephone officine + encodage caracteres PDF
- Lot 5: ecran point detaille entree/sortie (REST, filtres, exports)
- Lot 6: outils de diagnostic suggestion

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yHXmXEhxfoN5Bxw7wEXKj
</commit_message>
<xml_diff>
--- a/docs/CAHIER_DE_RECETTES.xlsx
+++ b/docs/CAHIER_DE_RECETTES.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Synthèse" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lot 1 - Annulation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lot 2 - Suggestion" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lot 1 - Modif vente" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lot 2 - Moteur suggestion" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Lot 3 - Tel tiers-payant" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lot 4 - Tel officine" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Lot 4 - Tel officine + PDF" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Lot 5 - Ecran E-S" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Lot 6 - Outils suggestion" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,11 +507,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
@@ -519,7 +520,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CAHIER DE RECETTES — PRESTIGE</t>
+          <t>CAHIER DE RECETTES — PRESTIGE (v2.0)</t>
         </is>
       </c>
     </row>
@@ -555,7 +556,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>5 lots de corrections et évolutions</t>
+          <t>6 lots — corrections, refonte écran entrée/sortie, outils suggestion</t>
         </is>
       </c>
     </row>
@@ -567,7 +568,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -579,204 +580,258 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0 (remplace la 1.0 : intègre les retours de recette et les évolutions suggestion/vente)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Légende des statuts :</t>
+          <t>Pré-requis de déploiement :</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>- Build : mvn package (JDK 11) doit produire prestige.war ; poi-4.1.1 / poi-ooxml-4.1.1 présents dans WEB-INF/lib</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>- Base : la migration Flyway V6.3.1 (index t_warehouse) s'exécute au premier démarrage — peut prendre du temps sur une grosse table</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>- Comptes : A avec privilège P_BT_ANNULER_VENTE, B (caissière) sans ce privilège</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>- Paramètres &gt; Identification pharmacie renseignés (téléphone principal + autres téléphones)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Légende :</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Résultat conforme au résultat attendu</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Conforme au résultat attendu</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>KO</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Résultat non conforme (à détailler en Observations)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Non conforme (détailler en Observations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Non applicable / non testé</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Intitulé</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Testeur</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Attribution de l'annulation + privilège API</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Modification de vente : attribution annulation, privilège API, suppression copie sur Retour</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Suggestion de réapprovisionnement</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Moteur de suggestion de réapprovisionnement (règles métier)</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Téléphone tiers-payant dans les éditions</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Téléphone officine (facture, proforma, BL)</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Téléphone officine + encodage des documents PDF</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Refonte écran Point détaillé entrée/sortie</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Écran Point détaillé entrée/sortie (refonte REST)</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Écran Suggestion : diagnostic, rattrapage, consultation</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Décision de mise en production :</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>☐ Validée      ☐ Validée avec réserves      ☐ Refusée</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Validé par :</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Fonction :</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Date :</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="15">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:E3"/>
+    <mergeCell ref="A13:E13"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:E6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C15:C19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C21:C26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,NA"</formula1>
     </dataValidation>
   </dataValidations>
@@ -790,7 +845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -804,11 +859,11 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOT 1 — Attribution de l'annulation + privilège API</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>LOT 1 — Modification de vente clôturée</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Objectif</t>
@@ -816,11 +871,11 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>L'annulation automatique de l'ancienne vente (parcours Ventes terminées → Modifier) doit être attribuée à l'utilisateur ayant lancé la modification, pas au caissier qui clôture la copie. L'annulation directe via l'API doit exiger le privilège P_BT_ANNULER_VENTE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>Attribution correcte de l'annulation automatique (à l'utilisateur qui a lancé la modification), contrôle du privilège P_BT_ANNULER_VENTE sur l'annulation directe, et suppression de la copie quand on quitte la modification par Retour (fin des ventes en attente orphelines).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Fichiers concernés</t>
@@ -828,7 +883,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>SalesServiceImpl.java (clôture assurance et comptant), SalesRessource.java, VenteRessource.java</t>
+          <t>SalesServiceImpl.java, SalesRessource.java, VenteRessource.java, VenteCtr.js</t>
         </is>
       </c>
     </row>
@@ -877,9 +932,9 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>1. Utilisateur A ouvre une vente terminée → Modifier.
+          <t>1. Utilisateur A : Ventes terminées &gt; Modifier.
 2. A modifie les articles et clôture la copie.
-3. Consulter la liste des ventes annulées.</t>
+3. Consulter les ventes annulées.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -898,15 +953,14 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Reprise par une caissière différente (comptant)</t>
+          <t>Copie mise en ATTENTE puis clôturée par une caissière (comptant)</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>1. A ouvre une vente comptant terminée → Modifier → Retour.
-2. Connexion avec la caissière B.
-3. B ouvre la vente en attente, supprime/ajoute des produits, clôture.
-4. Consulter les ventes annulées.</t>
+          <t>1. A : Modifier &gt; bouton ATTENTE (la copie est conservée volontairement).
+2. Caissière B reprend la vente en attente, change les articles, clôture.
+3. Consulter les ventes annulées.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -930,7 +984,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Idem TC1.2 mais sur une vente assurance (tiers-payant).</t>
+          <t>Idem TC1.2 sur une vente assurance (tiers-payant).</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -949,23 +1003,23 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Clôture de la copie autorisée sans droit d'annulation</t>
+          <t>Clôture de la copie non bloquée par le privilège</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>La caissière B (sans P_BT_ANNULER_VENTE) clôture la copie issue de « Modifier ».</t>
+          <t>La caissière B (sans P_BT_ANNULER_VENTE) clôture la copie.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>La clôture aboutit normalement (non bloquée : l'annulation est un effet automatique).</t>
+          <t>La clôture aboutit (l'annulation de l'originale est un effet automatique, pas une annulation directe).</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
       <c r="F10" s="11" t="inlineStr"/>
     </row>
-    <row r="11" ht="70" customHeight="1">
+    <row r="11" ht="55" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>TC1.5</t>
@@ -973,17 +1027,17 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Annulation directe via API SANS privilège</t>
+          <t>Annulation directe API sans privilège</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Avec le compte B (sans P_BT_ANNULER_VENTE), appeler l'annulation directe d'une vente (v1/vente/annulation/{id} ou v2/vente/annulation/{id}).</t>
+          <t>Compte B : appeler v1/vente/annulation/{id} (ou v2).</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Opération refusée (« Vous n'avez pas l'autorisation d'annuler une vente ») ; la vente n'est pas annulée.</t>
+          <t>Refus « Vous n'avez pas l'autorisation d'annuler une vente » ; la vente n'est pas annulée.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr"/>
@@ -997,12 +1051,12 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Annulation directe via API AVEC privilège</t>
+          <t>Annulation directe API avec privilège</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Avec le compte A (avec P_BT_ANNULER_VENTE), annuler directement une vente.</t>
+          <t>Compte A : annuler directement une vente.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1026,34 +1080,134 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Réaliser une vente comptant classique et la clôturer.</t>
+          <t>Vente comptant classique, clôture.</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>La vente se clôture normalement, aucune annulation parasite.</t>
+          <t>Clôture normale, aucune annulation parasite.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr"/>
       <c r="F13" s="7" t="inlineStr"/>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TC1.8</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>RETOUR supprime la copie</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>1. Ventes terminées &gt; Modifier (la copie s'ouvre).
+2. Cliquer RETOUR.
+3. Consulter les ventes en attente.</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Aucune vente en attente issue de la modification : la copie a été supprimée.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>TC1.9</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>La vente originale redevient modifiable après Retour</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Après TC1.8, rouvrir Ventes terminées et cliquer Modifier sur la même vente.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>La modification s'ouvre normalement (nouvelle copie créée).</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="55" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>TC1.10</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>ATTENTE conserve la copie</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>1. Modifier une vente clôturée.
+2. Cliquer ATTENTE (pas Retour).
+3. Consulter les ventes en attente.</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>La copie est bien présente en vente en attente (conservation volontaire).</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>TC1.11</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Garde-fou : l'endpoint copie refuse une vente normale</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Appeler DELETE /api/v1/vente/copie/{id} avec l'id d'une vente clôturée ou d'une prévente ordinaire.</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Refus « Cette vente n'est pas une copie de modification en cours » ; rien n'est supprimé.</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Recette réalisée par :</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Date :</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Verdict :</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1062,10 +1216,10 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E7:E13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E7:E17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,NA"</formula1>
     </dataValidation>
-    <dataValidation sqref="F15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,NA"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1079,7 +1233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1093,11 +1247,11 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOT 2 — Suggestion de réapprovisionnement</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>LOT 2 — Moteur de suggestion de réapprovisionnement</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Objectif</t>
@@ -1105,11 +1259,11 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Un produit vendu atteignant son seuil doit remonter en suggestion, sauf s'il est réellement dans une commande active (is_Process/pharma) ou une suggestion active. Une ancienne commande non active ne doit plus bloquer, et le contrôle « déjà en suggestion » doit fonctionner (paramètre JPQL ?4 corrigé).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>Règles métier validées : (1) produit dans le processus de commande -&gt; jamais suggéré ; (2) produit dans une suggestion AUTO non traitée + revente -&gt; quantité mise à jour ; (3) suggestion ouverte (pending) + revente -&gt; NOUVELLE suggestion auto ; (4) commande supprimée -&gt; produit re-suggérable. Et l'énigme résolue : les vieilles commandes zombies ne bloquent plus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Fichiers concernés</t>
@@ -1153,7 +1307,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="70" customHeight="1">
+    <row r="7" ht="55" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>TC2.1</t>
@@ -1166,13 +1320,12 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>1. Produit actif, suggérable, non déconditionné, seuil défini, sans commande ni suggestion.
-2. Le vendre jusqu'au seuil.</t>
+          <t>Produit actif, suggérable, seuil défini, hors commande/suggestion. Le vendre jusqu'au seuil.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Le produit remonte en suggestion (suggestions auto).</t>
+          <t>Le produit apparaît dans une suggestion auto.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr"/>
@@ -1186,18 +1339,17 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Produit déjà dans une commande active</t>
+          <t>Produit dans une commande active</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>1. Produit présent dans une commande is_Process ou pharma (non reçue).
-2. Le vendre au seuil.</t>
+          <t>Produit dans une commande en cours (is_Process/pharma, non reçue). Le vendre au seuil.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Le produit n'est pas re-suggéré (blocage légitime).</t>
+          <t>Pas de suggestion (blocage légitime), peu importe le nombre de ventes.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr"/>
@@ -1211,18 +1363,17 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Ancienne commande non active (bug corrigé)</t>
+          <t>Vieille commande zombie (l'énigme d'origine)</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>1. Produit avec ligne t_order_detail rattachée à une commande recu=false mais dont le statut n'est pas is_Process/pharma.
-2. Le vendre au seuil.</t>
+          <t>Produit avec ligne t_order_detail rattachée à une commande recu=false mais non active (fermée/incohérente). Le vendre au seuil.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Le produit remonte bien en suggestion (l'ancienne commande ne bloque plus).</t>
+          <t>Le produit est suggéré : la commande zombie ne bloque plus.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr"/>
@@ -1236,24 +1387,23 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Produit déjà dans une suggestion active</t>
+          <t>Déjà dans une suggestion AUTO non traitée</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>1. Produit déjà dans une suggestion auto ou is_Process.
-2. Le vendre à nouveau au seuil.</t>
+          <t>Produit dans une suggestion auto. Le revendre.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Pas de doublon : la quantité de la ligne existante est mise à jour, aucune nouvelle suggestion créée.</t>
+          <t>PAS de doublon : la quantité de sa ligne est mise à jour dans la suggestion existante.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
       <c r="F10" s="11" t="inlineStr"/>
     </row>
-    <row r="11" ht="40" customHeight="1">
+    <row r="11" ht="55" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>TC2.5</t>
@@ -1261,23 +1411,24 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Non-régression : produit non éligible</t>
+          <t>Suggestion prise en main (pending) puis revente</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Vendre au seuil un produit inactif, ou déconditionné, ou non suggérable.</t>
+          <t>1. Ouvrir la suggestion auto via Modifier (elle passe en pending).
+2. Revendre un de ses produits au seuil.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Le produit n'est jamais suggéré.</t>
+          <t>Une NOUVELLE suggestion auto est créée avec ce produit (comportement métier historique).</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr"/>
       <c r="F11" s="7" t="inlineStr"/>
     </row>
-    <row r="12" ht="55" customHeight="1">
+    <row r="12" ht="40" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>TC2.6</t>
@@ -1285,101 +1436,121 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Vérification technique (logs)</t>
+          <t>Suppression de la commande en cours</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Après une session de ventes déclenchant des suggestions, consulter les logs applicatifs.</t>
+          <t>Supprimer la commande en cours contenant le produit, puis le vendre au seuil.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Aucune exception de paramètre JPQL non lié (?4) ; erreurs éventuelles tracées en WARNING au lieu d'être muettes.</t>
+          <t>Le produit est à nouveau suggéré.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr"/>
       <c r="F12" s="11" t="inlineStr"/>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Requête SQL diagnostic (a) — Produits au seuil bloqués par une ligne de commande</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="165" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>SELECT f.lg_FAMILLE_ID, f.int_CIP, f.str_NAME, fs.int_NUMBER_AVAILABLE, f.int_SEUIL_MIN,
-       od.str_STATUT AS statut_detail, o.str_REF_ORDER, o.str_STATUT AS statut_commande, o.recu
-FROM t_famille f
-JOIN t_famille_stock fs ON fs.lg_FAMILLE_ID = f.lg_FAMILLE_ID
-JOIN t_order_detail od ON od.lg_FAMILLE_ID = f.lg_FAMILLE_ID
-JOIN t_order o ON o.lg_ORDER_ID = od.lg_ORDER_ID
-WHERE f.str_STATUT = 'enable' AND COALESCE(f.bool_DECONDITIONNE,0) &lt;&gt; 1
-  AND COALESCE(f.bool_SUGGERABLE,1) = 1 AND f.int_SEUIL_MIN IS NOT NULL
-  AND fs.int_NUMBER_AVAILABLE &lt;= f.int_SEUIL_MIN
-ORDER BY o.dt_CREATED DESC, f.str_NAME;</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Requête SQL diagnostic (b) — Détail is_Process mais commande non active</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="165" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>SELECT f.lg_FAMILLE_ID, f.int_CIP, f.str_NAME, od.str_STATUT AS statut_detail,
-       o.str_REF_ORDER, o.str_STATUT AS statut_commande, o.recu
-FROM t_order_detail od
-JOIN t_order o ON o.lg_ORDER_ID = od.lg_ORDER_ID
-JOIN t_famille f ON f.lg_FAMILLE_ID = od.lg_FAMILLE_ID
-JOIN t_famille_stock fs ON fs.lg_FAMILLE_ID = f.lg_FAMILLE_ID
-WHERE od.str_STATUT = 'is_Process'
-  AND (o.str_STATUT NOT IN ('is_Process','pharma') OR o.str_STATUT IS NULL OR o.recu = TRUE)
-  AND f.int_SEUIL_MIN IS NOT NULL AND fs.int_NUMBER_AVAILABLE &lt;= f.int_SEUIL_MIN
-ORDER BY o.dt_CREATED DESC, f.str_NAME;</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>TC2.7</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Produit non éligible</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Vendre au seuil un produit inactif, déconditionné ou non suggérable.</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Jamais suggéré.</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TC2.8</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Vérification technique (logs)</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Après une session de ventes, consulter les logs serveur.</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Aucune exception JPQL (paramètre non lié) ; les erreurs éventuelles de ces contrôles sont loggées en WARNING.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Requête SQL de vérification de l'état des suggestions</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>-- Suggestions actives et anciennete des lignes (verification de l'etat des donnees)
+SELECT s.lg_SUGGESTION_ORDER_ID, s.str_STATUT, s.dt_CREATED, s.dt_UPDATED, COUNT(d.lg_SUGGESTION_ORDER_DETAILS_ID) AS nb_lignes
+FROM t_suggestion_order s
+LEFT JOIN t_suggestion_order_details d ON d.lg_SUGGESTION_ORDER_ID = s.lg_SUGGESTION_ORDER_ID
+WHERE d.str_STATUT IN ('auto', 'is_Process')
+GROUP BY s.lg_SUGGESTION_ORDER_ID, s.str_STATUT, s.dt_CREATED, s.dt_UPDATED
+ORDER BY s.dt_UPDATED ASC;</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Recette réalisée par :</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Date :</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Verdict :</t>
         </is>
       </c>
-      <c r="F21" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="5">
     <mergeCell ref="B4:F4"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E7:E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E7:E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,NA"</formula1>
     </dataValidation>
-    <dataValidation sqref="F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,NA"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1411,7 +1582,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Objectif</t>
@@ -1419,11 +1590,11 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Le numéro du tiers-payant/client (stocké dans le champ adresse) doit conserver son 0 initial dans les éditions (champ MATRO et paramètre P_CODE_POSTALE). Règle : un numéro local de 9 chiffres ne commençant pas par 0 est préfixé d'un 0 ; toute autre valeur est conservée (après trim).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>Le numéro du tiers-payant/client (champ adresse) conserve son 0 initial dans les éditions (MATRO, P_CODE_POSTALE). Règle : 9 chiffres ne commençant pas par 0 -&gt; préfixé ; toute autre valeur conservée (trim).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Fichiers concernés</t>
@@ -1431,7 +1602,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>StringUtils.normalizePhone, ReportDataSource.java, FactureProvisoire.java, InvoiceServlet.java, rest/report/pdf/Facture.java, 4 JSP d'édition de factures</t>
+          <t>StringUtils.normalizePhone, ReportDataSource, FactureProvisoire, InvoiceServlet, Facture, 4 JSP d'édition</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1656,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Édition affiche : 0708094545</t>
+          <t>Édition : 0708094545</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr"/>
@@ -1499,7 +1670,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Numéro local déjà correct</t>
+          <t>Numéro déjà correct</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -1509,13 +1680,13 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Édition affiche : 0708094545 (inchangé)</t>
+          <t>Édition : 0708094545 (inchangé)</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr"/>
       <c r="F8" s="11" t="inlineStr"/>
     </row>
-    <row r="9" ht="40" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>TC3.3</t>
@@ -1523,7 +1694,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Numéro international</t>
+          <t>International</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -1533,13 +1704,13 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Édition affiche : +2250708094545 (inchangé)</t>
+          <t>Édition : +2250708094545 (inchangé)</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr"/>
     </row>
-    <row r="10" ht="40" customHeight="1">
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
           <t>TC3.4</t>
@@ -1547,7 +1718,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Numéro avec espaces</t>
+          <t>Avec espaces</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -1557,7 +1728,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Édition affiche : 01 02 03 04 05 (inchangé)</t>
+          <t>Édition : 01 02 03 04 05 (inchangé)</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
@@ -1571,7 +1742,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Valeur vide</t>
+          <t>Vide</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -1595,12 +1766,12 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Rendu sur facture tiers-payant</t>
+          <t>Facture tiers-payant</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Générer une facture tiers-payant dont le tiers-payant a le téléphone 708094545.</t>
+          <t>Générer une facture d'un tiers-payant au téléphone 708094545.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1653,7 +1824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1667,11 +1838,11 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOT 4 — Téléphone officine (facture, proforma, bon de livraison)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>LOT 4 — Téléphone officine et encodage des documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Objectif</t>
@@ -1679,11 +1850,11 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Le téléphone de l'officine (Paramètres → Identification pharmacie) doit conserver son 0 initial, au format (+225) 07-08-09-45-45. Logique centralisée dans DateConverter.phoneNumberFormat, puis re-pointage des documents facture/proforma/BL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>Le téléphone de l'officine (Paramètres &gt; Identification pharmacie) conserve son 0 au format (+225) 07-08-09-45-45 sur facture, proforma et bon de livraison. Les caractères spéciaux (°, é, ô) des documents sont réparés (fini les « ï¿½ »).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Fichiers concernés</t>
@@ -1691,276 +1862,311 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>DateConverter.phoneNumberFormat, InvoiceServlet.java, ReportDataSource.java, ws_rp_facture_tiers_payant.jsp, ws_rp_print_all_invoices.jsp, group_invoice_pdf.jsp, ws_allinvoice_pdf.jsp, ws_generate_devis_pdf.jsp (proforma), bonlivraison/ws_generate_pdf.jsp</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Point de vigilance (hors régression) : un numéro officine stocké avec le préfixe +225 inclus (ex. +2250708094545) n'est pas reformaté et retombe sur l'indicatif seul — comportement identique à l'avant-correction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+          <t>DateConverter.phoneNumberFormat, InvoiceServlet, ReportDataSource, JSP factures/proforma/BL, ws_transaction.jsp</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Scénario</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Étapes</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Résultat attendu</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>TC4.1</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Facture — numéro avec 0</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Tel officine = 0708094545. Générer une facture PDF.</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Facture — tel avec 0</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Tel officine 0708094545. Générer une facture PDF.</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>En-tête : Tel: (+225) 07-08-09-45-45</t>
         </is>
       </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>TC4.2</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Facture — tel sans 0 en base</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Tel officine 708094545. Facture PDF.</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Tel: (+225) 07-08-09-45-45</t>
+        </is>
+      </c>
       <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>TC4.2</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Facture — numéro sans 0 en base</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>Tel officine = 708094545. Générer une facture PDF.</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>Tel: (+225) 07-08-09-45-45</t>
+      <c r="F8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>TC4.3</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Proforma / devis</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Tel officine 708094545. Proforma PDF.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>(+225) 07-08-09-45-45</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="11" t="inlineStr"/>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>TC4.3</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Proforma / devis</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Tel officine = 708094545. Générer une proforma PDF.</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>TC4.4</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Bon de livraison</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Tel officine 708094545. BL PDF.</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>(+225) 07-08-09-45-45</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>TC4.4</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Bon de livraison</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>Tel officine = 708094545. Générer un bon de livraison PDF.</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>(+225) 07-08-09-45-45</t>
+      <c r="F10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>TC4.5</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Ancien numéro 8 chiffres</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Tel officine 20304050. Facture PDF.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>(+225) 20-30-40-50 (inchangé)</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="11" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>TC4.5</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Ancien numéro à 8 chiffres</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Tel officine = 20304050. Générer une facture PDF.</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>(+225) 20-30-40-50 (inchangé)</t>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>TC4.6</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Autres téléphones (;)</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>strAUTRESPHONES = 708094545;0102030405. Facture PDF.</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>07-08-09-45-45 / 01-02-03-04-05</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>TC4.6</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>Autres téléphones (séparés par ;)</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>strAUTRESPHONES = 708094545;0102030405. Générer une facture PDF.</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>Chaque numéro avec son 0 : 07-08-09-45-45 / 01-02-03-04-05</t>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>TC4.7</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Non-régression ticket de caisse</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Imprimer un ticket.</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Ticket inchangé (hors périmètre, comme convenu).</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="11" t="inlineStr"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>TC4.7</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Non-régression — ticket de caisse</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Tel officine renseigné. Imprimer un ticket de caisse.</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Le ticket est inchangé (hors périmètre, comme convenu).</t>
+      <c r="F13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TC4.8</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Caractères spéciaux — factures</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Générer une facture PDF (tiers-payant).</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Plus aucun « ï¿½ » : FACTURE N°, RC N°, CC N°, CPT N°, Régime d'Imposition, Centre des Impôts s'affichent correctement.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15" ht="55" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>TC4.8</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Facture tiers-payant (les 2 corrections)</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>Officine = 708094545 ET tiers-payant = 708094545. Générer la facture tiers-payant.</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>Officine : (+225) 07-08-09-45-45 ; tiers-payant : 0708094545</t>
+      <c r="F14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>TC4.9</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Caractères spéciaux — BL et proforma</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Générer un bon de livraison et une proforma.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Accents corrects (é, ô, °) sur tout le document.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr"/>
-      <c r="F15" s="11" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>TC4.10</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Message écran famille</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Tenter de supprimer un article déjà utilisé (écran famille).</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Message « ...déjà été utilisé dans le système » avec accents corrects.</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="11" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Recette réalisée par :</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Date :</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Verdict :</t>
         </is>
       </c>
-      <c r="F17" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E8:E15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E7:E16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,NA"</formula1>
     </dataValidation>
-    <dataValidation sqref="F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,NA"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1974,7 +2180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1988,11 +2194,11 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOT 5 — Refonte écran Point détaillé entrée/sortie</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+          <t>LOT 5 — Écran Point détaillé entrée/sortie (refonte REST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Objectif</t>
@@ -2000,11 +2206,11 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Remplacer les 5 JSP historiques par l'API REST /api/v1/stock-movements : filtres combinables, exports Excel/CSV, créations inventaire/suggestion, sans régression. Fabricant retiré, grossiste visible, COMMANDE retiré, PERIME renommé « Saisie en périmés », AJUSTEMENT ajouté.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>API unique /api/v1/stock-movements ; type « Tous » par défaut ; dates du jour préremplies ; colonne Date = date du mouvement ; filtres combinables ; exports xlsx/csv ; créations inventaire/suggestion ; erreurs visibles (success=false + msg) ; performances (requêtes indexables + index Flyway V6.3.1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Fichiers concernés</t>
@@ -2012,7 +2218,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>StockMovementRessource.java, StockMovementDataHelper.java, StockMovementFilterDTO.java, SuiviDetailStockVenteManager.js, pom.xml (poi-ooxml)</t>
+          <t>StockMovementRessource/DataHelper, SuiviDetailStockVenteManager.js, pom.xml (poi 4.1.1), V6.3.1__indexes_warehouse_mouvements.sql</t>
         </is>
       </c>
     </row>
@@ -2048,7 +2254,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1">
+    <row r="7" ht="70" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>TC5.1</t>
@@ -2066,13 +2272,13 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Grille chargée sur ENTRÉE EN STOCK par défaut, sans erreur.</t>
+          <t>Type « Tous » sélectionné, dates du jour préremplies dans Date début et Date fin, données du jour (tous types) triées du plus récent au plus ancien.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr"/>
       <c r="F7" s="7" t="inlineStr"/>
     </row>
-    <row r="8" ht="40" customHeight="1">
+    <row r="8" ht="55" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>TC5.2</t>
@@ -2080,23 +2286,23 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Recherche texte</t>
+          <t>Colonne Date renseignée</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Saisir un CIP ou nom d'article puis Rechercher.</t>
+          <t>Filtre Entrée en stock, observer les colonnes.</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Seules les lignes correspondantes s'affichent.</t>
+          <t>Colonne Date = date du mouvement (plus jamais vide), colonne Heure = heure du mouvement.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr"/>
       <c r="F8" s="11" t="inlineStr"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="40" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>TC5.3</t>
@@ -2104,23 +2310,23 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Date début seule</t>
+          <t>Filtre Tous</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Renseigner uniquement la date de début.</t>
+          <t>Sélectionner « Tous » avec une période.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Filtre &gt;= date début appliqué.</t>
+          <t>Mouvements de tous types mélangés, tri chronologique décroissant.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="55" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
           <t>TC5.4</t>
@@ -2128,23 +2334,23 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Date fin seule</t>
+          <t>Types individuels</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Renseigner uniquement la date de fin.</t>
+          <t>Tester Entrée en stock, Saisie en périmés, Retour fournisseur, Vente, Ajustement.</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Filtre &lt;= date fin appliqué.</t>
+          <t>Chaque type renvoie ses mouvements ; COMMANDE n'existe plus ; libellé « Saisie en perimes » présent.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
       <c r="F10" s="11" t="inlineStr"/>
     </row>
-    <row r="11" ht="40" customHeight="1">
+    <row r="11" ht="55" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>TC5.5</t>
@@ -2152,23 +2358,23 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Période complète</t>
+          <t>Saisie de périmés visible</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Renseigner début et fin.</t>
+          <t>Faire une saisie en périmés (validée), puis filtre Saisie en périmés (dates du jour).</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Les deux bornes inclusives sont appliquées.</t>
+          <t>La saisie apparaît (y compris pour un produit sans grossiste).</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr"/>
       <c r="F11" s="7" t="inlineStr"/>
     </row>
-    <row r="12" ht="40" customHeight="1">
+    <row r="12" ht="55" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>TC5.6</t>
@@ -2176,23 +2382,23 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Filtre grossiste</t>
+          <t>Retour fournisseur visible</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Sélectionner un grossiste.</t>
+          <t>Saisir un retour fournisseur (même non validé en avoir), filtre Retour fournisseur.</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Résultats restreints au grossiste ; champ grossiste visible.</t>
+          <t>Le retour apparaît avec date, quantité, motif, grossiste, opérateur.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr"/>
       <c r="F12" s="11" t="inlineStr"/>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="40" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>TC5.7</t>
@@ -2200,23 +2406,23 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Filtre famille article</t>
+          <t>Historique des petites tables</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Sélectionner une famille article.</t>
+          <t>Vider les deux dates, filtre Retour fournisseur (ou Périmés/Ajustement).</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Résultats restreints à la famille.</t>
+          <t>Tout l'historique s'affiche (pas seulement le jour).</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr"/>
       <c r="F13" s="7" t="inlineStr"/>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="40" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
           <t>TC5.8</t>
@@ -2224,17 +2430,17 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Filtre emplacement / zone géo</t>
+          <t>Filtres combinables</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Sélectionner une zone.</t>
+          <t>Type + grossiste + famille article + zone + recherche + période.</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Résultats restreints à la zone.</t>
+          <t>Tous les filtres s'appliquent ensemble, sans erreur.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr"/>
@@ -2248,17 +2454,17 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Combinaison de tous les filtres</t>
+          <t>Grossiste sur les ventes</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Type + grossiste + famille + zone + recherche + période.</t>
+          <t>Type Vente + grossiste.</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Tous les filtres se combinent, aucun ignoré ni erreur.</t>
+          <t>Ventes des produits rattachés à ce grossiste (grossiste par défaut du produit).</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr"/>
@@ -2272,23 +2478,23 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Type ENTRÉE EN STOCK</t>
+          <t>Pagination conserve les filtres</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Sélectionner ce type.</t>
+          <t>Filtres actifs, changer de page.</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Lignes d'entrées en stock (mêmes colonnes qu'avant).</t>
+          <t>La page suivante conserve tous les filtres.</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr"/>
       <c r="F16" s="11" t="inlineStr"/>
     </row>
-    <row r="17" ht="40" customHeight="1">
+    <row r="17" ht="55" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>TC5.11</t>
@@ -2296,23 +2502,23 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Type Saisie en périmés</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Sélectionner ce type.</t>
+          <t>Mesurer le GET (réseau) sur Vente et Entrée en stock, dates du jour, après le premier démarrage (index créés).</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Libellé « Saisie en périmés » ; lignes de périmés remontent.</t>
+          <t>Temps de réponse nettement inférieur aux mesures initiales (3,5-6,7 s) ; pas de scan complet.</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr"/>
       <c r="F17" s="7" t="inlineStr"/>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="55" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
           <t>TC5.12</t>
@@ -2320,23 +2526,23 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Type Retour fournisseur</t>
+          <t>Erreurs visibles</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Sélectionner ce type.</t>
+          <t>En cas de filtre en échec (le cas échéant).</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Lignes de retours fournisseur.</t>
+          <t>La réponse porte success=false et un msg explicite (visible dans l'onglet réseau) — plus de faux « total: 0 ».</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr"/>
       <c r="F18" s="11" t="inlineStr"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="55" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>TC5.13</t>
@@ -2344,23 +2550,23 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Type Vente</t>
+          <t>Export Excel</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Sélectionner ce type.</t>
+          <t>Filtres actifs &gt; bouton Excel.</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Lignes de ventes.</t>
+          <t>Fichier .xlsx téléchargé (plus d'erreur 500 Date1904Support), toutes les lignes filtrées.</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr"/>
       <c r="F19" s="7" t="inlineStr"/>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="40" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>TC5.14</t>
@@ -2368,23 +2574,23 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Type Ajustement (nouveau)</t>
+          <t>Export CSV</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Sélectionner ce type.</t>
+          <t>Filtres actifs &gt; bouton CSV.</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Les produits ajustés remontent.</t>
+          <t>Fichier .csv (séparateur ;, accents corrects), toutes les lignes filtrées.</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr"/>
       <c r="F20" s="11" t="inlineStr"/>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="55" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t>TC5.15</t>
@@ -2392,23 +2598,23 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Type Commande retiré</t>
+          <t>Création d'inventaire (2 modes)</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Ouvrir la liste des types.</t>
+          <t>a) Cocher des lignes &gt; Inventaire. b) Sans cocher &gt; Inventaire.</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Le type COMMANDE n'apparaît plus.</t>
+          <t>a) inventaire avec les produits cochés ; b) avec tout le résultat filtré ; confirmation avant exécution.</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr"/>
       <c r="F21" s="7" t="inlineStr"/>
     </row>
-    <row r="22" ht="40" customHeight="1">
+    <row r="22" ht="55" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
           <t>TC5.16</t>
@@ -2416,23 +2622,23 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Filtre fabricant retiré</t>
+          <t>Création de suggestion (2 modes)</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Observer la barre de filtres.</t>
+          <t>Idem avec le bouton Suggestion.</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Le filtre fabricant n'apparaît plus et n'est plus envoyé.</t>
+          <t>Suggestion créée (regroupée par grossiste) ; produits sans grossiste ignorés proprement.</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr"/>
       <c r="F22" s="11" t="inlineStr"/>
     </row>
-    <row r="23" ht="55" customHeight="1">
+    <row r="23" ht="70" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>TC5.17</t>
@@ -2440,17 +2646,17 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Grossiste sur les ventes</t>
+          <t>Comparaison REST vs JSP</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Type Vente + un grossiste sélectionné.</t>
+          <t>Pour chaque type conservé, comparer total/lignes avec l'ancienne JSP sur plusieurs filtres.</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Ventes des produits rattachés à ce grossiste (grossiste par défaut) ; aucune erreur si produit sans grossiste.</t>
+          <t>Résultats identiques (aux évolutions volontaires près : Tous, Ajustement, colonnes complétées, retours non validés visibles).</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr"/>
@@ -2464,375 +2670,39 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Pagination conserve les filtres</t>
+          <t>Session expirée</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Appliquer des filtres puis changer de page.</t>
+          <t>Appeler l'API sans session.</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>La page suivante conserve tous les filtres (correction du bug de pagination).</t>
+          <t>Réponse d'échec propre (non connecté), pas d'erreur serveur.</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr"/>
       <c r="F24" s="11" t="inlineStr"/>
     </row>
-    <row r="25" ht="70" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>TC5.19</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Comparaison REST vs JSP</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Pour chaque type, comparer total et lignes entre l'ancienne JSP et la nouvelle API sur plusieurs jeux de filtres.</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Résultats identiques (aux évolutions volontaires près : Commande retiré, Ajustement ajouté, colonnes article complétées pour les périmés).</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr"/>
-      <c r="F25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="55" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>TC5.20</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>Export Excel (.xlsx)</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>Appliquer des filtres puis cliquer Excel.</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>Fichier .xlsx téléchargé avec TOUTES les lignes filtrées (pas la page courante).</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr"/>
-      <c r="F26" s="11" t="inlineStr"/>
-    </row>
-    <row r="27" ht="40" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>TC5.21</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Export CSV</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Appliquer des filtres puis cliquer CSV.</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Fichier .csv (séparateur ;, accents corrects) avec toutes les lignes filtrées.</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr"/>
-      <c r="F27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="40" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>TC5.22</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Exports reprennent les filtres</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>Modifier les filtres puis relancer un export.</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>L'export reflète exactement les filtres en cours.</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr"/>
-      <c r="F28" s="11" t="inlineStr"/>
-    </row>
-    <row r="29" ht="55" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>TC5.23</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Inventaire depuis sélection</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Cocher des lignes puis Inventaire → confirmer.</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Inventaire créé avec uniquement les produits cochés ; message du nombre pris en compte.</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr"/>
-      <c r="F29" s="7" t="inlineStr"/>
-    </row>
-    <row r="30" ht="40" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>TC5.24</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>Inventaire depuis tout le filtre</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>Sans rien cocher, Inventaire → confirmer.</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>Inventaire créé avec tous les produits du résultat filtré.</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr"/>
-      <c r="F30" s="11" t="inlineStr"/>
-    </row>
-    <row r="31" ht="40" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>TC5.25</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Suggestion depuis sélection</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Cocher des lignes puis Suggestion → confirmer.</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Suggestion créée pour les produits cochés (regroupés par grossiste).</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr"/>
-      <c r="F31" s="7" t="inlineStr"/>
-    </row>
-    <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>TC5.26</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>Suggestion depuis tout le filtre</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>Sans rien cocher, Suggestion → confirmer.</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>Suggestion créée pour tous les produits filtrés ayant un grossiste.</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr"/>
-      <c r="F32" s="11" t="inlineStr"/>
-    </row>
-    <row r="33" ht="55" customHeight="1">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>TC5.27</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Confirmation avant création</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Cliquer sur Inventaire ou Suggestion.</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>Une confirmation précise le périmètre (sélection ou tout le filtre) avant exécution.</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="inlineStr"/>
-      <c r="F33" s="7" t="inlineStr"/>
-    </row>
-    <row r="34" ht="55" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>TC5.28</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>Produits sans grossiste (suggestion)</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>Lancer une suggestion sur un lot contenant des produits sans grossiste par défaut.</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>Produits sans grossiste ignorés proprement ; message si aucun produit éligible.</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr"/>
-      <c r="F34" s="11" t="inlineStr"/>
-    </row>
-    <row r="35" ht="40" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>TC5.29</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Contrat de réponse REST</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>Interroger GET /api/v1/stock-movements?...</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>Réponse avec success, total et results (compatible grille ExtJS).</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="inlineStr"/>
-      <c r="F35" s="7" t="inlineStr"/>
-    </row>
-    <row r="36" ht="40" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>TC5.30</t>
-        </is>
-      </c>
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t>Bornes de dates</t>
-        </is>
-      </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
-          <t>Vérifier les résultats en limite de période.</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t>Dates &gt;= (00:00:00) et &lt;= (23:59:59), bornes incluses.</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr"/>
-      <c r="F36" s="11" t="inlineStr"/>
-    </row>
-    <row r="37" ht="40" customHeight="1">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>TC5.31</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Session expirée</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>Appeler l'API sans session valide.</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Réponse d'échec cohérente (non connecté), pas d'erreur serveur.</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="inlineStr"/>
-      <c r="F37" s="7" t="inlineStr"/>
-    </row>
-    <row r="38" ht="40" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>TC5.32</t>
-        </is>
-      </c>
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>Dépendance build</t>
-        </is>
-      </c>
-      <c r="C38" s="11" t="inlineStr">
-        <is>
-          <t>Compiler/packager le projet (mvn package).</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="inlineStr">
-        <is>
-          <t>Le build aboutit avec la dépendance poi-ooxml (export .xlsx).</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="inlineStr"/>
-      <c r="F38" s="11" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Recette réalisée par :</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Date :</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Verdict :</t>
         </is>
       </c>
-      <c r="F40" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2841,10 +2711,393 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E7:E38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E7:E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,NA"</formula1>
     </dataValidation>
-    <dataValidation sqref="F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"OK,KO,NA"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LOT 6 — Écran Suggestion : diagnostic, rattrapage, consultation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Objectif</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Fenêtre Diagnostic produit (pourquoi pas suggéré ?), liste des produits au seuil non suggérés (sans disable/delete), création de suggestion depuis le diagnostic (sélection multi-pages/multi-recherches ou tout), et consultation d'une suggestion en lecture seule (sans passage en pending).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Fichiers concernés</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>SuggestionImpl, SuggestionRessource, Suggestion_Manager.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Scénario</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Étapes</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Résultat attendu</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Observations</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>TC6.1</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Ouverture du diagnostic</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Écran Liste Suggestion &gt; bouton « Diagnostic produit ».</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Fenêtre avec champ de recherche, grille (coche, CIP, article, statut, stock, seuil, grossiste, diagnostic) et boutons.</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>TC6.2</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Recherche tous statuts</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Rechercher un produit en statut disable.</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Le produit est trouvé avec le diagnostic « Produit inactif (statut disable) : exclu de la suggestion ».</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>TC6.3</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Diagnostics explicites</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Rechercher des produits dans différents cas : seuil non atteint, en commande, sans grossiste, déjà en suggestion, sans blocage.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Chaque cas affiche sa cause exacte (avec stock/seuil/condition pour le seuil) ; « Aucun blocage : sera suggéré à la prochaine vente » en vert.</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>TC6.4</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Liste des produits au seuil non suggérés</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Bouton « Produits au seuil non suggérés ».</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Liste paginée des produits au seuil absents de toute suggestion auto active ; AUCUN produit disable ou delete dans la liste.</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>TC6.5</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Coches conservées multi-recherches / multi-pages</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>1. Rechercher A, cocher 2 produits.
+2. Rechercher B, cocher 1 produit.
+3. Ouvrir la liste des non-suggérés, page 2, cocher 1.
+4. Revenir sur la recherche A.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Les produits déjà cochés réapparaissent cochés ; le cumul (4) est conservé.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="70" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>TC6.6</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Créer suggestion — sélection</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Avec des produits cochés, bouton « Créer suggestion » &gt; confirmer.</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Message « X ajouté(s) sur Y traité(s) » ; les produits cochés SANS blocage sont dans la suggestion auto ; les bloqués sont ignorés ; les coches sont vidées.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="70" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>TC6.7</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Créer suggestion — tout le rattrapage</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Sans rien cocher, « Créer suggestion » &gt; confirmation « TOUS les produits au seuil non suggérés ».</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>L'arriéré part en suggestion ; la liste des non-suggérés se vide de ces produits ; la grille des suggestions se rafraîchit.</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TC6.8</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Cohérence avec le moteur</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Vérifier la quantité d'un produit ajouté via le diagnostic.</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Même quantité que si la suggestion avait été déclenchée par une vente (même calcul de réappro, même grossiste).</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="70" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>TC6.9</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Consultation en lecture seule (Voir)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Icône « Voir » (liste) sur une suggestion AUTO &gt; consulter &gt; fermer &gt; vérifier le statut.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Contenu affiché (CIP, article, stock, seuil, qté, prix) avec filtre/pagination ; le statut de la suggestion reste AUTO (pas de passage en pending).</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="55" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>TC6.10</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Voir n'interrompt pas l'alimentation auto</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Après TC6.9, vendre au seuil un produit du même grossiste.</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>La suggestion auto consultée continue d'être alimentée (nouvelle ligne ou quantité mise à jour).</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>TC6.11</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Modifier passe toujours en pending</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Icône « Modifier » (crayon) sur une suggestion auto.</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>L'écran de gestion s'ouvre et la suggestion passe en pending (comportement historique conservé).</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Recette réalisée par :</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Date :</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Verdict :</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:F3"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="E7:E17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"OK,KO,NA"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,NA"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>